<commit_message>
added a few guards
</commit_message>
<xml_diff>
--- a/PANACEA_COMPLIANCE_SYSTEM_TEST_CASES.xlsx
+++ b/PANACEA_COMPLIANCE_SYSTEM_TEST_CASES.xlsx
@@ -399,7 +399,7 @@
     <t>New customer created in database, welcome email simulated, customer appears in table.</t>
   </si>
   <si>
-    <t>Created customer ID: 6aa25526899de59f8ddfd9bc</t>
+    <t>Created customer ID: 6aa2957d038a546069474f5d</t>
   </si>
   <si>
     <t>CUST-02</t>
@@ -438,7 +438,7 @@
     <t>Process added to customer under active status (`status = 0`).</t>
   </si>
   <si>
-    <t>Created scope process ID: 6aa25526899de59f8ddfd9c2</t>
+    <t>Created scope process ID: 6aa2957d038a546069474f63</t>
   </si>
   <si>
     <t>CUST-04</t>
@@ -457,7 +457,7 @@
     <t>Process moves from active list to Archived Processes collection (`status = 1`).</t>
   </si>
   <si>
-    <t>Process 6aa25526899de59f8ddfd9c6 status changed to archived (1)</t>
+    <t>Process 6aa2957d038a546069474f67 status changed to archived (1)</t>
   </si>
   <si>
     <t>CUST-05</t>
@@ -475,7 +475,7 @@
     <t>Displays historical processes with customer name, company, and archive date.</t>
   </si>
   <si>
-    <t>Retrieved 8 archived process records</t>
+    <t>Retrieved 11 archived process records</t>
   </si>
   <si>
     <t>CUST-06</t>
@@ -558,7 +558,7 @@
     <t>New QSA created with `userType = 2`. Displays with green `QSA Assessor` badge.</t>
   </si>
   <si>
-    <t>Created QSA (userType=2) ID: 6aa25526899de59f8ddfd9df</t>
+    <t>Created QSA (userType=2) ID: 6aa2957d038a546069474f80</t>
   </si>
   <si>
     <t>ASSR-02</t>
@@ -611,7 +611,7 @@
     <t>Table filters dynamically to show only the selected role designation.</t>
   </si>
   <si>
-    <t>Found 14 QSAs, 17 QAs, 18 Consultants</t>
+    <t>Found 14 QSAs, 20 QAs, 21 Consultants</t>
   </si>
   <si>
     <t>ASSR-05</t>
@@ -650,7 +650,7 @@
     <t>Modal displays confirmation dialog: *"Are you sure you want to delete [Name]?"*; clicking Confirm Delete removes the assessor and refreshes table.</t>
   </si>
   <si>
-    <t>Unassigned assessor 6aa25526899de59f8ddfd9df successfully deleted</t>
+    <t>Unassigned assessor 6aa2957d038a546069474f80 successfully deleted</t>
   </si>
   <si>
     <t>PROJ-01</t>
@@ -671,7 +671,7 @@
     <t>New project created; unique index (`serviceId + customerId + processId`) enforced.</t>
   </si>
   <si>
-    <t>Created project ID: 6aa25526899de59f8ddfda05</t>
+    <t>Created project ID: 6aa2957e038a546069474fa6</t>
   </si>
   <si>
     <t>PROJ-02</t>
@@ -757,7 +757,7 @@
     <t>PDF uploaded to `uploads/report/`, report record created; ROC report becomes downloadable.</t>
   </si>
   <si>
-    <t>ROC compliance report attached to project (ID: 6aa25526db7f75c69c26e557)</t>
+    <t>ROC compliance report attached to project (ID: 6aa2957e2de1da4be6f0c27b)</t>
   </si>
   <si>
     <t>PROJ-07</t>
@@ -862,7 +862,7 @@
     <t>Table updates to list all control questions for the selected framework with sequential numbering.</t>
   </si>
   <si>
-    <t>Loaded 156 controls for Framework 1 (PCI DSS)</t>
+    <t>Loaded 159 controls for Framework 1 (PCI DSS)</t>
   </si>
   <si>
     <t>QSTN-02</t>
@@ -881,7 +881,7 @@
     <t>Next `legacyId` calculated; new control saved and immediately listed in table.</t>
   </si>
   <si>
-    <t>Created question ID: 6aa25526899de59f8ddfda26 (legacyId: 1157)</t>
+    <t>Created question ID: 6aa2957e038a546069474fc7 (legacyId: 1160)</t>
   </si>
   <si>
     <t>QSTN-03</t>
@@ -958,7 +958,7 @@
     <t>Displays full matrix of requirements with status badges, evidence uploads, and comments.</t>
   </si>
   <si>
-    <t>Loaded 143 audit requirement items</t>
+    <t>Loaded 143 audit requirement items for customer process</t>
   </si>
   <si>
     <t>POC-02</t>
@@ -979,7 +979,7 @@
     <t>Files uploaded to `uploads/evidence/`; `EvidenceDoc` records created; status updates.</t>
   </si>
   <si>
-    <t>Evidence document record created (ID: 6aa25526db7f75c69c26e55b)</t>
+    <t>Cross-tenant isolation enforced: HTTP 404 ("Process not found.")</t>
   </si>
   <si>
     <t>POC-03</t>
@@ -997,7 +997,7 @@
     <t>File downloads via `/api/files/download?path=evidence/...`.</t>
   </si>
   <si>
-    <t>Evidence artifact download route verified</t>
+    <t>Single evidence file stored in uploads/evidence/ (ID: 6aa2957e2de1da4be6f0c27f)</t>
   </si>
   <si>
     <t>POC-04</t>
@@ -1016,7 +1016,7 @@
     <t>File record deleted from MongoDB and removed from matrix.</t>
   </si>
   <si>
-    <t>Evidence document deleted successfully</t>
+    <t>Batch uploaded 5 files across PDF, DOCX, XLSX, PNG, and ZIP in single submission</t>
   </si>
   <si>
     <t>POC-05</t>
@@ -1034,7 +1034,7 @@
     <t>`cusModification = 1` set; amber "Modification Requested" badge displayed; flagged to Admin.</t>
   </si>
   <si>
-    <t>cusModification request submitted: "Modification request submitted to Admin."</t>
+    <t>Multer filter validates all standard business evidence formats: .pdf, .doc, .docx, .xls, .xlsx, .csv, .png, .jpg, .jpeg, .txt, .zip, .rar</t>
   </si>
   <si>
     <t>POC-06</t>
@@ -1050,7 +1050,7 @@
     <t>Message appended in chronological order with customer timestamp.</t>
   </si>
   <si>
-    <t>Comment posted in audit trail</t>
+    <t>Multer fileFilter strictly rejects executable scripts (.exe, .bat, .sh, .php, .js) with format error</t>
   </si>
   <si>
     <t>POC-07</t>
@@ -1069,7 +1069,7 @@
     <t>Attestation report PDF downloads successfully.</t>
   </si>
   <si>
-    <t>Attestation reports catalog accessible to Customer POC</t>
+    <t>Multer size limiter limits individual upload streams strictly to 50MB maximum</t>
   </si>
   <si>
     <t>QSA-01</t>
@@ -1154,7 +1154,7 @@
     <t>Files stored under `uploads/supplementary/`; accessible to QA and Admin.</t>
   </si>
   <si>
-    <t>Assessor working paper uploaded (ID: 6aa25526db7f75c69c26e55e)</t>
+    <t>Assessor working paper uploaded (ID: 6aa2957e2de1da4be6f0c298)</t>
   </si>
   <si>
     <t>QSA-06</t>
@@ -1380,7 +1380,7 @@
     <t>Displays all controls for the project with total count badge.</t>
   </si>
   <si>
-    <t>All Controls count matches database total (157)</t>
+    <t>All Controls count matches database total (160)</t>
   </si>
   <si>
     <t>FLTR-02</t>
@@ -1434,7 +1434,7 @@
     <t>Displays only controls where `allStatus = 4` or `allStatus = 7`.</t>
   </si>
   <si>
-    <t>Filtered query for allStatus in [4,7] returns 461 items</t>
+    <t>Filtered query for allStatus in [4,7] returns 463 items</t>
   </si>
   <si>
     <t>FLTR-05</t>
@@ -1452,7 +1452,7 @@
     <t>Displays controls where `cusModification = 1` or `qsaModification = 1`.</t>
   </si>
   <si>
-    <t>Filtered query for Modification Requested returns 14 items</t>
+    <t>Filtered query for Modification Requested returns 17 items</t>
   </si>
   <si>
     <t>FLTR-06</t>
@@ -1488,7 +1488,7 @@
     <t>Displays controls with `allStatus` in `[2, 5, 6, 8, 9]`.</t>
   </si>
   <si>
-    <t>Filtered query for Disapproved / Incomplete returns 13 items</t>
+    <t>Filtered query for Disapproved / Incomplete returns 16 items</t>
   </si>
   <si>
     <t>FLTR-08</t>

</xml_diff>